<commit_message>
Add build 17 log file analyzer
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -1,26 +1,174 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8010" tabRatio="500"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Tracker" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Cert Study Plan" sheetId="3" r:id="rId3"/>
-  </sheets>
-  <calcPr calcId="145621" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Template/>
+  <TotalTime>0</TotalTime>
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>3</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="3" baseType="lpstr">
+      <vt:lpstr>Tracker</vt:lpstr>
+      <vt:lpstr>Summary</vt:lpstr>
+      <vt:lpstr>Cert Study Plan</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>14.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <cp:lastModifiedBy>Legedia legend</cp:lastModifiedBy>
+  <cp:revision>0</cp:revision>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-06-17T18:18:02Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-06-28T23:07:50Z</dcterms:modified>
+  <dc:language>en-US</dc:language>
+</cp:coreProperties>
+</file>
+
+<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
+<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <c r="C49" i="2" l="1"/>
+  <c r="B49" i="2"/>
+  <c r="C48" i="2"/>
+  <c r="B48" i="2"/>
+  <c r="C47" i="2"/>
+  <c r="B47" i="2"/>
+  <c r="C46" i="2"/>
+  <c r="B46" i="2"/>
+  <c r="C45" i="2"/>
+  <c r="B45" i="2"/>
+  <c r="C44" i="2"/>
+  <c r="B44" i="2"/>
+  <c r="C43" i="2"/>
+  <c r="B43" i="2"/>
+  <c r="C42" i="2"/>
+  <c r="B42" i="2"/>
+  <c r="C41" i="2"/>
+  <c r="B41" i="2"/>
+  <c r="C40" i="2"/>
+  <c r="B40" i="2"/>
+  <c r="C39" i="2"/>
+  <c r="B39" i="2"/>
+  <c r="C38" i="2"/>
+  <c r="B38" i="2"/>
+  <c r="C37" i="2"/>
+  <c r="B37" i="2"/>
+  <c r="C36" i="2"/>
+  <c r="B36" i="2"/>
+  <c r="C35" i="2"/>
+  <c r="B35" i="2"/>
+  <c r="C34" i="2"/>
+  <c r="B34" i="2"/>
+  <c r="C33" i="2"/>
+  <c r="B33" i="2"/>
+  <c r="C32" i="2"/>
+  <c r="B32" i="2"/>
+  <c r="C31" i="2"/>
+  <c r="B31" i="2"/>
+  <c r="C30" i="2"/>
+  <c r="B30" i="2"/>
+  <c r="C29" i="2"/>
+  <c r="B29" i="2"/>
+  <c r="C28" i="2"/>
+  <c r="B28" i="2"/>
+  <c r="C27" i="2"/>
+  <c r="B27" i="2"/>
+  <c r="C26" i="2"/>
+  <c r="B26" i="2"/>
+  <c r="C25" i="2"/>
+  <c r="B25" i="2"/>
+  <c r="C24" i="2"/>
+  <c r="B24" i="2"/>
+  <c r="C23" i="2"/>
+  <c r="B23" i="2"/>
+  <c r="C22" i="2"/>
+  <c r="B22" i="2"/>
+  <c r="C21" i="2"/>
+  <c r="B21" i="2"/>
+  <c r="C20" i="2"/>
+  <c r="B20" i="2"/>
+  <c r="C19" i="2"/>
+  <c r="B19" i="2"/>
+  <c r="C18" i="2"/>
+  <c r="B18" i="2"/>
+  <c r="C17" i="2"/>
+  <c r="B17" i="2"/>
+  <c r="C16" i="2"/>
+  <c r="B16" i="2"/>
+  <c r="C15" i="2"/>
+  <c r="B15" i="2"/>
+  <c r="C14" i="2"/>
+  <c r="B14" i="2"/>
+  <c r="C13" i="2"/>
+  <c r="B13" i="2"/>
+  <c r="C12" i="2"/>
+  <c r="B12" i="2"/>
+  <c r="C11" i="2"/>
+  <c r="B11" i="2"/>
+  <c r="B6" i="2"/>
+  <c r="B7" i="2" s="1"/>
+  <c r="B5" i="2"/>
+  <c r="B4" i="2"/>
+  <c r="B3" i="2"/>
+  <c r="D40" i="2" l="1"/>
+  <c r="D34" i="2"/>
+  <c r="D45" i="2"/>
+  <c r="D44" i="2"/>
+  <c r="D46" i="2"/>
+  <c r="D29" i="2"/>
+  <c r="D35" i="2"/>
+  <c r="D41" i="2"/>
+  <c r="D47" i="2"/>
+  <c r="D27" i="2"/>
+  <c r="D16" i="2"/>
+  <c r="D22" i="2"/>
+  <c r="D28" i="2"/>
+  <c r="D32" i="2"/>
+  <c r="D17" i="2"/>
+  <c r="D26" i="2"/>
+  <c r="D23" i="2"/>
+  <c r="D33" i="2"/>
+  <c r="D15" i="2"/>
+  <c r="D21" i="2"/>
+  <c r="D39" i="2"/>
+  <c r="D38" i="2"/>
+  <c r="D12" i="2"/>
+  <c r="D18" i="2"/>
+  <c r="D24" i="2"/>
+  <c r="D30" i="2"/>
+  <c r="D36" i="2"/>
+  <c r="D42" i="2"/>
+  <c r="D48" i="2"/>
+  <c r="D14" i="2"/>
+  <c r="D20" i="2"/>
+  <c r="D11" i="2"/>
+  <c r="D13" i="2"/>
+  <c r="D19" i="2"/>
+  <c r="D25" i="2"/>
+  <c r="D31" i="2"/>
+  <c r="D37" i="2"/>
+  <c r="D43" i="2"/>
+  <c r="D49" i="2"/>
+</calcChain>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="595">
   <si>
     <t>Build #</t>
@@ -1810,7 +1958,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
@@ -2093,7 +2241,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -2270,7 +2418,28 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8010" tabRatio="500"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Tracker" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" r:id="rId2"/>
+    <sheet name="Cert Study Plan" sheetId="3" r:id="rId3"/>
+  </sheets>
+  <calcPr calcId="145621" iterateDelta="1E-4"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I247"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2886,13 +3055,27 @@
       <c r="D18" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>539</v>
-      </c>
-      <c r="F18" s="3"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
       <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/log-file-analyzer-ruby</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Multi-format Ruby CLI with batch analysis, per-file auto detection, time-window filtering, time-bucket summaries, YAML config defaults, CSV/JSON export, and direct file output.</t>
+        </is>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
@@ -7726,7 +7909,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D49"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8474,7 +8657,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Sync builds 17-19 and fix tracker audits
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -2495,23 +2495,23 @@
       <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-06-06</t>
         </is>
       </c>
       <c r="G2" s="5"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/expense-tracker</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Depth: Expanded</t>
         </is>
@@ -2530,23 +2530,23 @@
       <c r="D3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
       <c r="G3" s="5"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/Async-News-Aggregator</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Depth: Expanded</t>
         </is>
@@ -2565,23 +2565,23 @@
       <c r="D4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
       <c r="G4" s="5"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/Sales-Dashboard</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2600,23 +2600,23 @@
       <c r="D5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
       <c r="G5" s="5"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/file-organizer</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Depth: Expanded</t>
         </is>
@@ -2635,23 +2635,23 @@
       <c r="D6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
       <c r="G6" s="5"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/chat-server</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2670,23 +2670,23 @@
       <c r="D7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>2026-06-12</t>
         </is>
       </c>
       <c r="G7" s="5"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/House-price-predictor</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2705,23 +2705,23 @@
       <c r="D8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
       <c r="G8" s="5"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/Dev-toolkit</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Depth: Expanded</t>
         </is>
@@ -2740,23 +2740,23 @@
       <c r="D9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
       <c r="G9" s="5"/>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/Python-testing</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2775,23 +2775,23 @@
       <c r="D10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
       <c r="G10" s="5"/>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/Kanban-Board-Vanilla-JS</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2810,23 +2810,23 @@
       <c r="D11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
       <c r="G11" s="5"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/Typed-Task-Manager</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2845,23 +2845,23 @@
       <c r="D12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
       <c r="G12" s="5"/>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/music-player-es-modules</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2880,23 +2880,23 @@
       <c r="D13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
       <c r="G13" s="5"/>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/github-profile-viewer-vanilla-js</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2915,23 +2915,23 @@
       <c r="D14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/string-utils-jest</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Depth: Expanded</t>
         </is>
@@ -2950,23 +2950,23 @@
       <c r="D15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
       <c r="G15" s="5"/>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/php-contact-form-backend</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Depth: Deep</t>
         </is>
@@ -2985,23 +2985,23 @@
       <c r="D16" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
       <c r="G16" s="5"/>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/url-shortener-api</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Depth: Expanded</t>
         </is>
@@ -3020,23 +3020,23 @@
       <c r="D17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
       <c r="G17" s="5"/>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>https://github.com/breakingthebot/file-duplicate-finder-rust</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Depth: Expanded</t>
         </is>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G18" s="5"/>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Depth: Deep | Multi-format Ruby CLI with batch analysis, per-file auto detection, time-window filtering, time-bucket summaries, YAML config defaults, CSV/JSON export, and direct file output.</t>
+          <t>Depth: Deep | Streaming Ruby CLI with common/JSON and gzip input, batch analysis, per-file auto detection, time-window filtering, threshold exits, comparison mode, trend buckets, YAML config defaults, packaged install flow, and CSV/JSON export.</t>
         </is>
       </c>
     </row>
@@ -3090,13 +3090,27 @@
       <c r="D19" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>539</v>
-      </c>
-      <c r="F19" s="3"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
       <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/library-catalog-java</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Depth: Expanded</t>
+        </is>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
@@ -3111,13 +3125,27 @@
       <c r="D20" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="3"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/budget-tracker-console-app</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Depth: Expanded</t>
+        </is>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">

</xml_diff>

<commit_message>
Sync build index through quick notes android app
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3132,7 +3132,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G20" s="5"/>
@@ -3160,13 +3160,27 @@
       <c r="D21" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="3"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
       <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/habit-tracker-ios-swiftui</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Depth: Deep</t>
+        </is>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
@@ -3181,13 +3195,27 @@
       <c r="D22" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="3"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/quick-notes-android-compose</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Kotlin Android notes app with Jetpack Compose Material 3, Room persistence, tags, archive/restore flows, search, sort, home screen widgets, accessibility polish, and automated UI regression coverage.</t>
+        </is>
+      </c>
     </row>
     <row r="23" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">

</xml_diff>

<commit_message>
Sync builds 22-23 from GitHub, fix build 21's push date
sync-github-builds flagged two public repos untracked in builds.json
(server-setup-script, hammerspoon-config) and a push-date drift on
build 21. Added both as builds 22-23 in actual push order, corrected
build 21's date to match its real GitHub push date, and updated the
tracker workbook to match. audit-builds and sync-github-builds both
pass clean (23/23/23, 0 GitHub drift).
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3202,7 +3202,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="G22" s="5"/>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Depth: Deep | Kotlin Android notes app with Jetpack Compose Material 3, Room persistence, tags, archive/restore flows, search, sort, home screen widgets, accessibility polish, and automated UI regression coverage.</t>
+          <t>Depth: Deep</t>
         </is>
       </c>
     </row>
@@ -3230,13 +3230,27 @@
       <c r="D23" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F23" s="3"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
       <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/server-setup-script</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Bash automation script: package-manager-agnostic dependency install/verify, env.conf generation, config templating, cron-scheduled health checks, systemd service generator, Slack/Discord/webhook notifications, dry-run mode, and fail-safe rollback with diagnostic archiving.</t>
+        </is>
+      </c>
     </row>
     <row r="24" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
@@ -3251,13 +3265,27 @@
       <c r="D24" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="3"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
       <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/hammerspoon-config</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Window halves/thirds/maximize/center hotkeys, move-to-next/previous-screen with proportional resize across different-resolution monitors, app focus/launch/hide toggle, and GitHub Actions CI running the Lua test suite.</t>
+        </is>
+      </c>
     </row>
     <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">

</xml_diff>

<commit_message>
Sync build 24 (SQL Analytics Query Library) from GitHub
sync-github-builds flagged sql-analytics-library as untracked. Added
it as build 24 with actual push date. audit-builds and
sync-github-builds both pass clean (24/24/24, 0 GitHub drift).
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3300,13 +3300,27 @@
       <c r="D25" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F25" s="3"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
       <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/sql-analytics-library</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Depth: Deep | 20-query analytical SQL library over a mock e-commerce SQLite DB: high-fidelity data generator (VIP/corporate discounts, inventory logs), query benchmarking/profiler, HTML portfolio dashboard, interactive SQL REPL shell, and pytest coverage.</t>
+        </is>
+      </c>
     </row>
     <row r="26" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">

</xml_diff>

<commit_message>
Assign real categories, add per-category badge colors, sync build 25
Every build previously had category="Languages" -- one undifferentiated
group across all 24 entries, making By Category dead weight. Reclassified
into 8 real categories (CLI Tools, Web Frontend, Backend & Networking,
Data & Analytics, Libraries & Packages, Desktop & Console Apps, Mobile
Apps, Automation & DevOps) based on what each build actually is, and
gave each its own badge color like technology badges already have.

Also synced build 25 (FlavorFind Recipe Finder), found untracked while
re-running sync-github-builds during this change.
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3335,13 +3335,27 @@
       <c r="D26" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F26" s="3"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
       <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/flavorfind-recipe-finder</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Recipe search/filter app with dietary restriction filters, custom recipe CRUD synced to localStorage, cook-mode step timers parsed via regex, and a shopping list aggregator that normalizes units and merges duplicate ingredients across recipes.</t>
+        </is>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">

</xml_diff>

<commit_message>
Fix build 23's push-date drift
hammerspoon-config's pushedAt moved when I pushed its CI version bump
just now, which sync-github-builds treats as drift on any commit --
even trivial follow-ups unrelated to the build's actual content. Worth
knowing: this'll recur any time a build repo gets a follow-up commit
after being indexed, since the check compares against the *current*
last-push timestamp, not the original one.
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3272,7 +3272,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G24" s="5"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Depth: Deep | Window halves/thirds/maximize/center hotkeys, move-to-next/previous-screen with proportional resize across different-resolution monitors, app focus/launch/hide toggle, and GitHub Actions CI running the Lua test suite.</t>
+          <t>Depth: Deep</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add builds 26-28 (portfolio-site, shopping cart, GitHub dashboard)
Reconciled builds.json against the real public GitHub repos: added the
three React builds that were live but unindexed, and fixed build 25's
push-date drift (flavorfind got a later follow-up push). GitHub sync
audit and local audit both pass clean at 28/28.
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3342,7 +3342,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G26" s="5"/>
@@ -3370,13 +3370,27 @@
       <c r="D27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" s="3"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/portfolio-site</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Four-page site (Home, Projects, Blog, Contact) deployed to Vercel with a real Formspree-backed contact form. Replaced a stale third-party GitHub contribution chart with a first-party recent-activity widget after confirming the old one undercounted. Added per-page SEO titles, a generated sitemap.xml/robots.txt, and a WCAG contrast + heading-hierarchy + skip-link accessibility pass across 24 iterations.</t>
+        </is>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
@@ -3391,13 +3405,27 @@
       <c r="D28" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E28" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F28" s="3"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/react-zustand-shopping-cart</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Zustand store with persist/partialize middleware so only real cart items survive a refresh, not transient UI state. Promo code system (percentage, flat, and free-shipping codes) with derived pricing getters so tax/shipping/discount math lives in one place. Toast notifications replaced a forced cart-drawer-open UX. Vitest + React Testing Library coverage across cartStore and toastStore.</t>
+        </is>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
@@ -3412,13 +3440,27 @@
       <c r="D29" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F29" s="3"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
       <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/github-dashboard-react-query</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Every fetch goes through useQuery instead of a hand-rolled useEffect+fetch, giving real caching, a distinct loading-vs-refetching state, and structured error handling for free. Pagination reads GitHub's real Link response header instead of guessing from the current page number. The repo detail route (react-router-dom) fires three independent queries in parallel (details, languages, commits) so one slow or failed query never blocks the rest of the page. Deployed to Vercel with a vercel.json SPA rewrite so deep-linked detail routes survive a refresh.</t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">

</xml_diff>

<commit_message>
Add builds #29-31: Next.js blog, Remix todo, mobile expense tracker
Reconciled builds.json against public GitHub repos via sync-github-builds:
three repos existed on GitHub but weren't indexed yet. Added via the
release-day workflow (builds.json, README, per-build pages, tracker
workbook). 286-builds-dashboard intentionally left unindexed (series
tooling, not a numbered build).
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3475,13 +3475,27 @@
       <c r="D30" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="3"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
       <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/nextjs-blog-platform</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Postgres-backed comments (Neon serverless driver) with per-IP rate limiting (hashed IPs, 5 writes/10min), self-service comment deletion via hashed delete tokens, and an admin override checked with a constant-time comparison. Optimistic comment submission via useOptimistic/useTransition. Post tags with a statically generated /tags/[tag] route (not a query param, to preserve SSG). GitHub Actions CI and component tests with jsdom.</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
@@ -3496,13 +3510,27 @@
       <c r="D31" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E31" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F31" s="3"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
       <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/remix-todo-build30</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Nested routes for viewing/editing a single todo, each with its own loader/action and 404 handling. Optimistic UI on toggle/delete via useFetcher on both the list and detail routes. Data layer swapped from a hand-rolled JSON file to SQLite (better-sqlite3) without changing any exported function signatures, so no route or test code needed to change. GitHub Actions CI plus a Playwright smoke test.</t>
+        </is>
+      </c>
     </row>
     <row r="32" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
@@ -3517,13 +3545,27 @@
       <c r="D32" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E32" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F32" s="3"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
       <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/expense-tracker-build31</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Depth: Standard | Iteration 1: Expense model with validation, an AsyncStorage-backed local storage service, and a single-screen Add Expense form plus list, with delete. Amounts stored as integer cents so future totals (e.g. a monthly chart) sum exactly. 15 Jest tests cover validation and storage CRUD.</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">

</xml_diff>

<commit_message>
Update build index: Add Build 36 (PulseMarket) and Build 37 (PulseFit) entries, update spreadsheets and README
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3213,7 +3213,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Depth: Deep</t>
+          <t>Depth: Deep | Kotlin Android notes app with Jetpack Compose Material 3, Room persistence, tags, archive/restore flows, search, sort, home screen widgets, accessibility polish, and automated UI regression coverage.</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Depth: Deep</t>
+          <t>Depth: Deep | Window halves/thirds/maximize/center hotkeys, move-to-next/previous-screen with proportional resize across different-resolution monitors, app focus/launch/hide toggle, and GitHub Actions CI running the Lua test suite.</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Depth: Standard | Iteration 1: Expense model with validation, an AsyncStorage-backed local storage service, and a single-screen Add Expense form plus list, with delete. Amounts stored as integer cents so future totals (e.g. a monthly chart) sum exactly. 15 Jest tests cover validation and storage CRUD.</t>
+          <t>Depth: Expanded | Iteration 1: Expense model with validation, an AsyncStorage-backed local storage service, and a single-screen Add Expense form plus list, with delete. Amounts stored as integer cents so future totals (e.g. a monthly chart) sum exactly. 15 Jest tests cover validation and storage CRUD.</t>
         </is>
       </c>
     </row>
@@ -3580,13 +3580,27 @@
       <c r="D33" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F33" s="3"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
       <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/syllabus-viewer-build32</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Features raw JSON payload uploading, schema structure validations, required reading checkbox checks, and dark theme variables toggle.</t>
+        </is>
+      </c>
     </row>
     <row r="34" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
@@ -3601,13 +3615,27 @@
       <c r="D34" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E34" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" s="3"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
       <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/admin-panel-build33</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Includes client-side auth state simulation, route protection guards, breadcrumbs state selectors, and lazy-loaded child route sub-bundles.</t>
+        </is>
+      </c>
     </row>
     <row r="35" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
@@ -3622,13 +3650,27 @@
       <c r="D35" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" s="3"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
       <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/realtime-search-rxjs</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Features debounced search, memory caching, error boundary resilience, combineLatest state filters, local storage search history suggestion blurs, and infinite scrolling IntersectionObserver paging.</t>
+        </is>
+      </c>
     </row>
     <row r="36" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
@@ -3643,13 +3685,27 @@
       <c r="D36" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E36" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F36" s="3"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
       <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/angular-material-dashboard</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Premium administrative layouts featuring status counters, sorting search data tables, responsive charts, and input forms using full Angular Material component models.</t>
+        </is>
+      </c>
     </row>
     <row r="37" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
@@ -3664,13 +3720,27 @@
       <c r="D37" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E37" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F37" s="3"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
       <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/angular-ngrx-store-ecommerce</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Features NgRx Store, Effects, Selectors, LocalStorage MetaReducer hydration, wishlist drawer grids, checkout step wizards, and Star Rating badges.</t>
+        </is>
+      </c>
     </row>
     <row r="38" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
@@ -3685,13 +3755,27 @@
       <c r="D38" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E38" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F38" s="3"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/pulsefit-tracker</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Depth: Deep | Configured standard PWA webmanifest configurations, offline Service Workers, expandable daily settings, SVG circular progress rings, rising hydration wave overlays, and vertical statistics graphs.</t>
+        </is>
+      </c>
     </row>
     <row r="39" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">

</xml_diff>

<commit_message>
Add Build 38 index and update project tracker Excel sheets
</commit_message>
<xml_diff>
--- a/reference/286-projects-tracker.xlsx
+++ b/reference/286-projects-tracker.xlsx
@@ -3790,12 +3790,22 @@
       <c r="D39" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E39" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F39" s="3"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://github.com/breakingthebot/movie-watchlist-vue</t>
+        </is>
+      </c>
       <c r="I39" s="5"/>
     </row>
     <row r="40" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>